<commit_message>
Added user inputs data, donwlaod, and upload files
</commit_message>
<xml_diff>
--- a/Forecasted Output/Toronto_user_forecast.xlsx
+++ b/Forecasted Output/Toronto_user_forecast.xlsx
@@ -7,14 +7,14 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Forecast" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>date</t>
   </si>
@@ -44,6 +44,39 @@
   </si>
   <si>
     <t>2026-04-05</t>
+  </si>
+  <si>
+    <t>2026-04-06</t>
+  </si>
+  <si>
+    <t>2026-04-07</t>
+  </si>
+  <si>
+    <t>2026-04-08</t>
+  </si>
+  <si>
+    <t>2026-04-09</t>
+  </si>
+  <si>
+    <t>2026-04-10</t>
+  </si>
+  <si>
+    <t>2026-04-11</t>
+  </si>
+  <si>
+    <t>2026-04-12</t>
+  </si>
+  <si>
+    <t>2026-04-13</t>
+  </si>
+  <si>
+    <t>2026-04-14</t>
+  </si>
+  <si>
+    <t>2026-04-15</t>
+  </si>
+  <si>
+    <t>2026-04-16</t>
   </si>
 </sst>
 </file>
@@ -401,7 +434,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -426,16 +459,16 @@
         <v>5</v>
       </c>
       <c r="B2">
-        <v>13603654.44327744</v>
+        <v>13740800.61721551</v>
       </c>
       <c r="C2">
-        <v>4762509.852145215</v>
+        <v>4791930.643892105</v>
       </c>
       <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
         <v>1</v>
-      </c>
-      <c r="E2">
-        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -443,16 +476,16 @@
         <v>6</v>
       </c>
       <c r="B3">
-        <v>13365585.06292188</v>
+        <v>13694152.47469736</v>
       </c>
       <c r="C3">
-        <v>4714132.428130514</v>
+        <v>4805652.872110896</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>1.7</v>
       </c>
       <c r="E3">
-        <v>6</v>
+        <v>18.3</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -460,16 +493,16 @@
         <v>7</v>
       </c>
       <c r="B4">
-        <v>13116473.91438502</v>
+        <v>11355056.52254985</v>
       </c>
       <c r="C4">
-        <v>4694636.67860976</v>
+        <v>4273179.202047387</v>
       </c>
       <c r="D4">
-        <v>3</v>
+        <v>11.5</v>
       </c>
       <c r="E4">
-        <v>6</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -477,16 +510,16 @@
         <v>8</v>
       </c>
       <c r="B5">
-        <v>12934789.89178094</v>
+        <v>13051937.27531798</v>
       </c>
       <c r="C5">
-        <v>4611063.325714975</v>
+        <v>4647778.825079892</v>
       </c>
       <c r="D5">
-        <v>4</v>
+        <v>4.3</v>
       </c>
       <c r="E5">
-        <v>6</v>
+        <v>15.1</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -494,16 +527,203 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <v>13385484.82389661</v>
+        <v>13454533.81227602</v>
       </c>
       <c r="C6">
-        <v>4222526.302884353</v>
+        <v>4252429.615769168</v>
       </c>
       <c r="D6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E6">
-        <v>6</v>
+        <v>20.9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>14486176.14298079</v>
+      </c>
+      <c r="C7">
+        <v>4139902.630148539</v>
+      </c>
+      <c r="D7">
+        <v>2.7</v>
+      </c>
+      <c r="E7">
+        <v>16.6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8">
+        <v>14496659.38691805</v>
+      </c>
+      <c r="C8">
+        <v>4783839.090529501</v>
+      </c>
+      <c r="D8">
+        <v>-0.8</v>
+      </c>
+      <c r="E8">
+        <v>16.7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9">
+        <v>13933281.16213918</v>
+      </c>
+      <c r="C9">
+        <v>4848312.66934912</v>
+      </c>
+      <c r="D9">
+        <v>0.1</v>
+      </c>
+      <c r="E9">
+        <v>11.4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10">
+        <v>12812712.00928662</v>
+      </c>
+      <c r="C10">
+        <v>4578152.00177919</v>
+      </c>
+      <c r="D10">
+        <v>4.3</v>
+      </c>
+      <c r="E10">
+        <v>6.1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11">
+        <v>11146072.37609085</v>
+      </c>
+      <c r="C11">
+        <v>4217067.615219884</v>
+      </c>
+      <c r="D11">
+        <v>11.9</v>
+      </c>
+      <c r="E11">
+        <v>14.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12">
+        <v>11915814.31531488</v>
+      </c>
+      <c r="C12">
+        <v>4368082.026161612</v>
+      </c>
+      <c r="D12">
+        <v>9</v>
+      </c>
+      <c r="E12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13">
+        <v>13224210.135478</v>
+      </c>
+      <c r="C13">
+        <v>4187167.265062185</v>
+      </c>
+      <c r="D13">
+        <v>6.1</v>
+      </c>
+      <c r="E13">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14">
+        <v>13052886.09626589</v>
+      </c>
+      <c r="C14">
+        <v>3782738.193622106</v>
+      </c>
+      <c r="D14">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="E14">
+        <v>11.5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15">
+        <v>10854983.37741056</v>
+      </c>
+      <c r="C15">
+        <v>3901006.604834848</v>
+      </c>
+      <c r="D15">
+        <v>14.5</v>
+      </c>
+      <c r="E15">
+        <v>19.1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16">
+        <v>13332821.44951183</v>
+      </c>
+      <c r="C16">
+        <v>4708678.48659599</v>
+      </c>
+      <c r="D16">
+        <v>3.4</v>
+      </c>
+      <c r="E16">
+        <v>20.8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17">
+        <v>13719340.29626417</v>
+      </c>
+      <c r="C17">
+        <v>4805873.491409699</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17">
+        <v>11.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Small fixes to the website before adding the interactive_user_validation
</commit_message>
<xml_diff>
--- a/Forecasted Output/Toronto_user_forecast.xlsx
+++ b/Forecasted Output/Toronto_user_forecast.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>date</t>
   </si>
@@ -29,51 +29,6 @@
   </si>
   <si>
     <t>wind_speed</t>
-  </si>
-  <si>
-    <t>2026-04-01</t>
-  </si>
-  <si>
-    <t>2026-04-02</t>
-  </si>
-  <si>
-    <t>2026-04-03</t>
-  </si>
-  <si>
-    <t>2026-04-04</t>
-  </si>
-  <si>
-    <t>2026-04-05</t>
-  </si>
-  <si>
-    <t>2026-04-06</t>
-  </si>
-  <si>
-    <t>2026-04-07</t>
-  </si>
-  <si>
-    <t>2026-04-08</t>
-  </si>
-  <si>
-    <t>2026-04-09</t>
-  </si>
-  <si>
-    <t>2026-04-10</t>
-  </si>
-  <si>
-    <t>2026-04-11</t>
-  </si>
-  <si>
-    <t>2026-04-12</t>
-  </si>
-  <si>
-    <t>2026-04-13</t>
-  </si>
-  <si>
-    <t>2026-04-14</t>
-  </si>
-  <si>
-    <t>2026-04-15</t>
   </si>
   <si>
     <t>2026-04-16</t>
@@ -434,7 +389,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -459,271 +414,16 @@
         <v>5</v>
       </c>
       <c r="B2">
-        <v>13740800.61721551</v>
+        <v>11331164.93361063</v>
       </c>
       <c r="C2">
-        <v>4791930.643892105</v>
+        <v>4209111.073102198</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E2">
         <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3">
-        <v>13694152.47469736</v>
-      </c>
-      <c r="C3">
-        <v>4805652.872110896</v>
-      </c>
-      <c r="D3">
-        <v>1.7</v>
-      </c>
-      <c r="E3">
-        <v>18.3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4">
-        <v>11355056.52254985</v>
-      </c>
-      <c r="C4">
-        <v>4273179.202047387</v>
-      </c>
-      <c r="D4">
-        <v>11.5</v>
-      </c>
-      <c r="E4">
-        <v>19.9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5">
-        <v>13051937.27531798</v>
-      </c>
-      <c r="C5">
-        <v>4647778.825079892</v>
-      </c>
-      <c r="D5">
-        <v>4.3</v>
-      </c>
-      <c r="E5">
-        <v>15.1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6">
-        <v>13454533.81227602</v>
-      </c>
-      <c r="C6">
-        <v>4252429.615769168</v>
-      </c>
-      <c r="D6">
-        <v>6</v>
-      </c>
-      <c r="E6">
-        <v>20.9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7">
-        <v>14486176.14298079</v>
-      </c>
-      <c r="C7">
-        <v>4139902.630148539</v>
-      </c>
-      <c r="D7">
-        <v>2.7</v>
-      </c>
-      <c r="E7">
-        <v>16.6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8">
-        <v>14496659.38691805</v>
-      </c>
-      <c r="C8">
-        <v>4783839.090529501</v>
-      </c>
-      <c r="D8">
-        <v>-0.8</v>
-      </c>
-      <c r="E8">
-        <v>16.7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9">
-        <v>13933281.16213918</v>
-      </c>
-      <c r="C9">
-        <v>4848312.66934912</v>
-      </c>
-      <c r="D9">
-        <v>0.1</v>
-      </c>
-      <c r="E9">
-        <v>11.4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10">
-        <v>12812712.00928662</v>
-      </c>
-      <c r="C10">
-        <v>4578152.00177919</v>
-      </c>
-      <c r="D10">
-        <v>4.3</v>
-      </c>
-      <c r="E10">
-        <v>6.1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5">
-      <c r="A11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11">
-        <v>11146072.37609085</v>
-      </c>
-      <c r="C11">
-        <v>4217067.615219884</v>
-      </c>
-      <c r="D11">
-        <v>11.9</v>
-      </c>
-      <c r="E11">
-        <v>14.5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" t="s">
-        <v>15</v>
-      </c>
-      <c r="B12">
-        <v>11915814.31531488</v>
-      </c>
-      <c r="C12">
-        <v>4368082.026161612</v>
-      </c>
-      <c r="D12">
-        <v>9</v>
-      </c>
-      <c r="E12">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5">
-      <c r="A13" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13">
-        <v>13224210.135478</v>
-      </c>
-      <c r="C13">
-        <v>4187167.265062185</v>
-      </c>
-      <c r="D13">
-        <v>6.1</v>
-      </c>
-      <c r="E13">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="A14" t="s">
-        <v>17</v>
-      </c>
-      <c r="B14">
-        <v>13052886.09626589</v>
-      </c>
-      <c r="C14">
-        <v>3782738.193622106</v>
-      </c>
-      <c r="D14">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="E14">
-        <v>11.5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5">
-      <c r="A15" t="s">
-        <v>18</v>
-      </c>
-      <c r="B15">
-        <v>10854983.37741056</v>
-      </c>
-      <c r="C15">
-        <v>3901006.604834848</v>
-      </c>
-      <c r="D15">
-        <v>14.5</v>
-      </c>
-      <c r="E15">
-        <v>19.1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5">
-      <c r="A16" t="s">
-        <v>19</v>
-      </c>
-      <c r="B16">
-        <v>13332821.44951183</v>
-      </c>
-      <c r="C16">
-        <v>4708678.48659599</v>
-      </c>
-      <c r="D16">
-        <v>3.4</v>
-      </c>
-      <c r="E16">
-        <v>20.8</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5">
-      <c r="A17" t="s">
-        <v>20</v>
-      </c>
-      <c r="B17">
-        <v>13719340.29626417</v>
-      </c>
-      <c r="C17">
-        <v>4805873.491409699</v>
-      </c>
-      <c r="D17">
-        <v>1</v>
-      </c>
-      <c r="E17">
-        <v>11.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>